<commit_message>
feat: update frontend components, training data, dictionary and feedback analytics
</commit_message>
<xml_diff>
--- a/lunyoro-translator/backend/feedback/feedback_analytics.xlsx
+++ b/lunyoro-translator/backend/feedback/feedback_analytics.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1056,6 +1056,155 @@
         </is>
       </c>
       <c r="K13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-11T16:06:14.174903</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>en-&gt;lun</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>animals and people</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>enyamaiswa n'abantu</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>different meaning</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-11T16:06:17.779987</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>en-&gt;lun</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>nllb</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>animals and people</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ebisoro n'abantu</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>different meaning</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-11T16:27:59.023811</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>en-&gt;lun</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>people and animals</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>abantu n'ebisoro</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>both_models_correct</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1094,7 +1243,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -1104,7 +1253,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -1114,7 +1263,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -1134,7 +1283,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>58.3</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7">
@@ -1181,10 +1330,10 @@
     <row r="2">
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
+        <v>46.7</v>
       </c>
     </row>
     <row r="3">
@@ -1194,7 +1343,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
         <v>33.3</v>
@@ -1203,27 +1352,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>both</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>8.300000000000001</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>none</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>8.300000000000001</v>
+        <v>6.7</v>
       </c>
     </row>
   </sheetData>
@@ -1259,13 +1408,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>context</t>
+          <t>both_models_correct</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1275,17 +1424,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>spelling</t>
+          <t>context</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>both_models_wrong</t>
+          <t>spelling</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1295,7 +1444,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>both_models_correct</t>
+          <t>both_models_wrong</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1313,7 +1462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1352,6 +1501,14 @@
         <v>2</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>